<commit_message>
account for unavailable couriers
</commit_message>
<xml_diff>
--- a/sample_data/sample_dataset.xlsx
+++ b/sample_data/sample_dataset.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,16 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>permanent_unavailable</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>outsourced_unavailable</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>productivity_per_courier</t>
         </is>
       </c>
@@ -459,7 +469,7 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>44927.375</v>
+        <v>46235.375</v>
       </c>
       <c r="C2" t="n">
         <v>1020</v>
@@ -471,6 +481,12 @@
         <v>4</v>
       </c>
       <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -481,7 +497,7 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>44928.75</v>
+        <v>46236.75</v>
       </c>
       <c r="C3" t="n">
         <v>980</v>
@@ -493,6 +509,12 @@
         <v>5</v>
       </c>
       <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
         <v>12</v>
       </c>
     </row>
@@ -503,7 +525,7 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>44929.375</v>
+        <v>46266.375</v>
       </c>
       <c r="C4" t="n">
         <v>1100</v>
@@ -515,6 +537,12 @@
         <v>6</v>
       </c>
       <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
         <v>15</v>
       </c>
     </row>
@@ -525,7 +553,7 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>44930.75</v>
+        <v>46267.75</v>
       </c>
       <c r="C5" t="n">
         <v>1050</v>
@@ -537,6 +565,12 @@
         <v>5</v>
       </c>
       <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
         <v>11</v>
       </c>
     </row>

</xml_diff>